<commit_message>
solución en pagado del capítulo 4 que corrije el error que daba al editar un registro de la tabla. solución en borrar movimiento, para que regrese a su estado original el estatus_evento
</commit_message>
<xml_diff>
--- a/public/PresupuestoInicial/PRESUPUESTO INICIAL INGRESOS 2024 ACTUALIZADO 18-06-2024 .xlsx
+++ b/public/PresupuestoInicial/PRESUPUESTO INICIAL INGRESOS 2024 ACTUALIZADO 18-06-2024 .xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27813"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\btrujillo\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SAC-IPE\public\PresupuestoInicial\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C6C4E1B-A6F0-4F81-99D8-353EB07333D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADE58E62-A297-433B-81FF-90C94C9E4F0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="822" xr2:uid="{9539A8D9-1841-4346-A922-0009B4A42F3E}"/>
   </bookViews>
@@ -283,9 +283,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="44" formatCode="_-&quot;$&quot;* #,##0.00_-;\-&quot;$&quot;* #,##0.00_-;_-&quot;$&quot;* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -442,7 +442,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="22">
@@ -533,9 +533,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -573,7 +573,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -679,7 +679,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -821,7 +821,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -830,7 +830,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E34018DD-ECDB-49CC-B8B4-8192DBA1B262}">
   <dimension ref="A1:T24"/>
-  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="6" style="2" bestFit="1" customWidth="1"/>
@@ -844,7 +844,7 @@
     <col min="21" max="16384" width="11.42578125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" ht="48" thickBot="1">
+    <row r="1" spans="1:20" ht="48" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
@@ -906,7 +906,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="2" spans="1:20" s="6" customFormat="1" ht="25.5">
+    <row r="2" spans="1:20" s="6" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>20</v>
       </c>
@@ -969,7 +969,7 @@
         <v>78493723.840000004</v>
       </c>
     </row>
-    <row r="3" spans="1:20" s="6" customFormat="1" ht="25.5">
+    <row r="3" spans="1:20" s="6" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>20</v>
       </c>
@@ -1032,7 +1032,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:20" s="6" customFormat="1" ht="25.5">
+    <row r="4" spans="1:20" s="6" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>20</v>
       </c>
@@ -1095,7 +1095,7 @@
         <v>130822872.73999999</v>
       </c>
     </row>
-    <row r="5" spans="1:20" s="6" customFormat="1" ht="25.5">
+    <row r="5" spans="1:20" s="6" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>20</v>
       </c>
@@ -1158,7 +1158,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="6" customFormat="1" ht="25.5">
+    <row r="6" spans="1:20" s="6" customFormat="1" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>20</v>
       </c>
@@ -1221,7 +1221,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:20" ht="25.5">
+    <row r="7" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>33</v>
       </c>
@@ -1284,7 +1284,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:20" ht="25.5">
+    <row r="8" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>36</v>
       </c>
@@ -1347,7 +1347,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:20" ht="25.5">
+    <row r="9" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>39</v>
       </c>
@@ -1410,7 +1410,7 @@
         <v>5450</v>
       </c>
     </row>
-    <row r="10" spans="1:20" ht="25.5">
+    <row r="10" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>42</v>
       </c>
@@ -1473,7 +1473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:20" ht="25.5">
+    <row r="11" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>42</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>2134560</v>
       </c>
     </row>
-    <row r="12" spans="1:20" ht="25.5">
+    <row r="12" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>47</v>
       </c>
@@ -1599,7 +1599,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:20" ht="25.5">
+    <row r="13" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>50</v>
       </c>
@@ -1662,7 +1662,7 @@
         <v>27754.15</v>
       </c>
     </row>
-    <row r="14" spans="1:20" ht="25.5">
+    <row r="14" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>53</v>
       </c>
@@ -1725,7 +1725,7 @@
         <v>5500</v>
       </c>
     </row>
-    <row r="15" spans="1:20" ht="25.5">
+    <row r="15" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>33</v>
       </c>
@@ -1788,7 +1788,7 @@
         <v>1331.33</v>
       </c>
     </row>
-    <row r="16" spans="1:20" ht="25.5">
+    <row r="16" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>58</v>
       </c>
@@ -1851,7 +1851,7 @@
         <v>46580371.969999999</v>
       </c>
     </row>
-    <row r="17" spans="1:20" ht="25.5">
+    <row r="17" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>61</v>
       </c>
@@ -1914,7 +1914,7 @@
         <v>982007.1</v>
       </c>
     </row>
-    <row r="18" spans="1:20" ht="25.5">
+    <row r="18" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>64</v>
       </c>
@@ -1977,7 +1977,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:20" ht="25.5">
+    <row r="19" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>67</v>
       </c>
@@ -2040,7 +2040,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="25.5">
+    <row r="20" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>20</v>
       </c>
@@ -2102,7 +2102,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="30">
+    <row r="21" spans="1:20" ht="30" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>67</v>
       </c>
@@ -2165,7 +2165,7 @@
         <v>333333748</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="25.5">
+    <row r="22" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>67</v>
       </c>
@@ -2228,7 +2228,7 @@
         <v>28654113</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="25.5">
+    <row r="23" spans="1:20" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>33</v>
       </c>
@@ -2291,11 +2291,8 @@
         <v>8583334</v>
       </c>
     </row>
-    <row r="24" spans="1:20">
-      <c r="H24" s="10">
-        <f>SUM(H2:H23)</f>
-        <v>10965299525</v>
-      </c>
+    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="H24" s="10"/>
       <c r="I24" s="10"/>
       <c r="J24" s="10"/>
       <c r="K24" s="10"/>

</xml_diff>